<commit_message>
make separate file for sites and improve accuracy than before
</commit_message>
<xml_diff>
--- a/uploads/result-Test.xlsx.xlsx
+++ b/uploads/result-Test.xlsx.xlsx
@@ -410,7 +410,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="str">
-        <v>https://www.ebay.co.uk/itm/326784589677</v>
+        <v>https://www.ebay.co.uk/itm/326758544855</v>
       </c>
       <c r="B2" t="str">
         <v>ebay.co.uk</v>
@@ -422,12 +422,12 @@
         <v>Working</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-04-29T09:54:54.099Z</v>
+        <v>2026-05-05T05:18:56.564Z</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
-        <v>https://www.ebay.co.uk/itm/326758544855</v>
+        <v>https://www.ebay.co.uk/itm/326784589677</v>
       </c>
       <c r="B3" t="str">
         <v>ebay.co.uk</v>
@@ -439,7 +439,7 @@
         <v>Working</v>
       </c>
       <c r="E3" t="str">
-        <v>2026-04-29T09:54:54.112Z</v>
+        <v>2026-05-05T05:18:56.676Z</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -456,7 +456,7 @@
         <v>Working</v>
       </c>
       <c r="E4" t="str">
-        <v>2026-04-29T09:54:57.077Z</v>
+        <v>2026-05-05T05:19:00.731Z</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -473,7 +473,7 @@
         <v>Working</v>
       </c>
       <c r="E5" t="str">
-        <v>2026-04-29T09:54:57.182Z</v>
+        <v>2026-05-05T05:19:00.785Z</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -490,7 +490,7 @@
         <v>Not Found</v>
       </c>
       <c r="E6" t="str">
-        <v>2026-04-29T09:54:58.371Z</v>
+        <v>2026-05-05T05:19:02.034Z</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -507,7 +507,7 @@
         <v>Not Found</v>
       </c>
       <c r="E7" t="str">
-        <v>2026-04-29T09:54:59.455Z</v>
+        <v>2026-05-05T05:19:03.001Z</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -524,7 +524,7 @@
         <v>Working</v>
       </c>
       <c r="E8" t="str">
-        <v>2026-04-29T09:54:59.964Z</v>
+        <v>2026-05-05T05:19:03.376Z</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -541,7 +541,7 @@
         <v>Not Found</v>
       </c>
       <c r="E9" t="str">
-        <v>2026-04-29T09:55:00.554Z</v>
+        <v>2026-05-05T05:19:04.152Z</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -558,7 +558,7 @@
         <v>Not Found</v>
       </c>
       <c r="E10" t="str">
-        <v>2026-04-29T09:55:01.576Z</v>
+        <v>2026-05-05T05:19:05.292Z</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -575,12 +575,12 @@
         <v>Working</v>
       </c>
       <c r="E11" t="str">
-        <v>2026-04-29T09:55:02.867Z</v>
+        <v>2026-05-05T05:19:06.392Z</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
-        <v>https://www.ebay.co.uk/itm/186988099473</v>
+        <v>https://www.ebay.co.uk/itm/187558058326</v>
       </c>
       <c r="B12" t="str">
         <v>ebay.co.uk</v>
@@ -592,12 +592,12 @@
         <v>Not Found</v>
       </c>
       <c r="E12" t="str">
-        <v>2026-04-29T09:55:03.995Z</v>
+        <v>2026-05-05T05:19:07.596Z</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
-        <v>https://www.ebay.co.uk/itm/187558058326</v>
+        <v>https://www.ebay.co.uk/itm/186988099473</v>
       </c>
       <c r="B13" t="str">
         <v>ebay.co.uk</v>
@@ -609,12 +609,12 @@
         <v>Not Found</v>
       </c>
       <c r="E13" t="str">
-        <v>2026-04-29T09:55:04.075Z</v>
+        <v>2026-05-05T05:19:07.669Z</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="str">
-        <v>https://www.ebay.co.uk/itm/187557614314</v>
+        <v>https://www.ebay.co.uk/itm/187558063088</v>
       </c>
       <c r="B14" t="str">
         <v>ebay.co.uk</v>
@@ -626,12 +626,12 @@
         <v>Not Found</v>
       </c>
       <c r="E14" t="str">
-        <v>2026-04-29T09:55:05.104Z</v>
+        <v>2026-05-05T05:19:08.675Z</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="str">
-        <v>https://www.ebay.co.uk/itm/187558063088</v>
+        <v>https://www.ebay.co.uk/itm/187557614314</v>
       </c>
       <c r="B15" t="str">
         <v>ebay.co.uk</v>
@@ -643,7 +643,7 @@
         <v>Not Found</v>
       </c>
       <c r="E15" t="str">
-        <v>2026-04-29T09:55:05.114Z</v>
+        <v>2026-05-05T05:19:08.952Z</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -660,7 +660,7 @@
         <v>Not Found</v>
       </c>
       <c r="E16" t="str">
-        <v>2026-04-29T09:55:06.278Z</v>
+        <v>2026-05-05T05:19:10.059Z</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -677,7 +677,7 @@
         <v>Not Found</v>
       </c>
       <c r="E17" t="str">
-        <v>2026-04-29T09:55:07.453Z</v>
+        <v>2026-05-05T05:19:11.411Z</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -694,7 +694,7 @@
         <v>Working</v>
       </c>
       <c r="E18" t="str">
-        <v>2026-04-29T09:55:07.942Z</v>
+        <v>2026-05-05T05:19:12.067Z</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -711,7 +711,7 @@
         <v>Not Found</v>
       </c>
       <c r="E19" t="str">
-        <v>2026-04-29T09:55:08.625Z</v>
+        <v>2026-05-05T05:19:12.596Z</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -728,7 +728,7 @@
         <v>Not Found</v>
       </c>
       <c r="E20" t="str">
-        <v>2026-04-29T09:55:09.049Z</v>
+        <v>2026-05-05T05:19:13.427Z</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -745,7 +745,7 @@
         <v>Not Found</v>
       </c>
       <c r="E21" t="str">
-        <v>2026-04-29T09:55:09.839Z</v>
+        <v>2026-05-05T05:19:14.040Z</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -762,7 +762,7 @@
         <v>Working</v>
       </c>
       <c r="E22" t="str">
-        <v>2026-04-29T09:55:12.853Z</v>
+        <v>2026-05-05T05:19:17.088Z</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -779,7 +779,7 @@
         <v>Working</v>
       </c>
       <c r="E23" t="str">
-        <v>2026-04-29T09:55:12.981Z</v>
+        <v>2026-05-05T05:19:17.092Z</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -796,7 +796,7 @@
         <v>Working</v>
       </c>
       <c r="E24" t="str">
-        <v>2026-04-29T09:55:16.054Z</v>
+        <v>2026-05-05T05:19:20.362Z</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -813,7 +813,7 @@
         <v>Working</v>
       </c>
       <c r="E25" t="str">
-        <v>2026-04-29T09:55:16.063Z</v>
+        <v>2026-05-05T05:19:20.462Z</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -830,7 +830,7 @@
         <v>Working</v>
       </c>
       <c r="E26" t="str">
-        <v>2026-04-29T09:55:19.058Z</v>
+        <v>2026-05-05T05:19:23.091Z</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -847,7 +847,7 @@
         <v>Working</v>
       </c>
       <c r="E27" t="str">
-        <v>2026-04-29T09:55:19.084Z</v>
+        <v>2026-05-05T05:19:23.339Z</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -864,7 +864,7 @@
         <v>Working</v>
       </c>
       <c r="E28" t="str">
-        <v>2026-04-29T09:55:22.287Z</v>
+        <v>2026-05-05T05:19:26.331Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>